<commit_message>
Updated BRA_grids model - 2025-09-19 18:21
</commit_message>
<xml_diff>
--- a/VerveStacks_BRA_grids/SuppXLS/trades/scentrade__trade_links.xlsx
+++ b/VerveStacks_BRA_grids/SuppXLS/trades/scentrade__trade_links.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_BRA_grids\SuppXLS\trades\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{97670242-97EC-4E25-A56A-7E7B9F21D795}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4EFA5189-CAF8-4C5D-A505-70A9A0817253}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{D0910A7D-AE40-4D01-A05D-B825C42786B4}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{7064F54A-1DC8-46BE-A94B-6B4E3D573E85}"/>
   </bookViews>
   <sheets>
     <sheet name="grid_links" sheetId="1" r:id="rId1"/>
@@ -3763,7 +3763,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79F02641-336D-4B8C-81E9-A90630167819}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28C3F2AF-9758-487F-B3E5-39A8FE86A188}">
   <dimension ref="B3:L489"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>